<commit_message>
Add hot update files for webpack and purchases page
- Created new hot update JavaScript files for the purchases page and various webpack configurations.
- Added corresponding hot update JSON files to track changes and dependencies.
- Implemented eval-source-map for development purposes, ensuring better debugging capabilities.
</commit_message>
<xml_diff>
--- a/New Microsoft Excel Worksheet.xlsx
+++ b/New Microsoft Excel Worksheet.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>PurchaseService.php</t>
   </si>
@@ -29,15 +29,28 @@
   </si>
   <si>
     <t>المشتريات:Purchase</t>
+  </si>
+  <si>
+    <t>php artisan optimize:clear</t>
+  </si>
+  <si>
+    <t>delete cash  &gt;&gt;&gt;&gt;&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -84,12 +97,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -396,7 +412,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="39.21875" customWidth="1"/>
@@ -404,45 +420,52 @@
     <col min="3" max="3" width="35.109375" customWidth="1"/>
     <col min="4" max="4" width="31.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="36.109375" customWidth="1"/>
+    <col min="6" max="6" width="41.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:6" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:6" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="1"/>
+      <c r="E2" s="2"/>
     </row>
-    <row r="3" spans="1:5" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="1:5" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:5" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="1:5" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="1:5" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:5" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="9" spans="1:5" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="1:5" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="1:5" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="12" spans="1:5" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="13" spans="1:5" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="1:5" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="15" spans="1:5" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="1:5" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:6" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="1:6" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:6" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:6" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:6" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:6" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="1:6" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="1:6" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="1:6" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="12" spans="1:6" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:6" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="1:6" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="15" spans="1:6" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:6" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="17" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="18" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="19" ht="32.4" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>